<commit_message>
Clarify project scope and complete workflow artifacts
</commit_message>
<xml_diff>
--- a/docs/excel-proof/losslens_synthetic_practice.xlsx
+++ b/docs/excel-proof/losslens_synthetic_practice.xlsx
@@ -10,15 +10,17 @@
     <sheet name="Start Here" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Events" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Cases" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Reconciliation" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="One Page Summary" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Actions" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Reconciliation" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="One Page Summary" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Start Here'!$A$1:$B$10</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Events'!$A$1:$J$14</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Cases'!$A$1:$R$3</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Reconciliation'!$A$1:$M$6</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'One Page Summary'!$A$1:$C$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Cases'!$A$1:$S$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Actions'!$A$1:$G$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Reconciliation'!$A$1:$M$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'One Page Summary'!$A$1:$C$10</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -175,9 +177,9 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Cases" displayName="Cases" ref="A1:R3" headerRowCount="1">
-  <autoFilter ref="A1:R3"/>
-  <tableColumns count="18">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Cases" displayName="Cases" ref="A1:S3" headerRowCount="1">
+  <autoFilter ref="A1:S3"/>
+  <tableColumns count="19">
     <tableColumn id="1" name="case_id"/>
     <tableColumn id="2" name="simulated"/>
     <tableColumn id="3" name="case_type"/>
@@ -196,13 +198,30 @@
     <tableColumn id="16" name="closed_at"/>
     <tableColumn id="17" name="open_age_days"/>
     <tableColumn id="18" name="closed_duration_days"/>
+    <tableColumn id="19" name="opened_week"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium4" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Reconciliation" displayName="Reconciliation" ref="A1:M6" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Actions" displayName="Actions" ref="A1:G3" headerRowCount="1">
+  <autoFilter ref="A1:G3"/>
+  <tableColumns count="7">
+    <tableColumn id="1" name="action_id"/>
+    <tableColumn id="2" name="case_id"/>
+    <tableColumn id="3" name="process_change"/>
+    <tableColumn id="4" name="owner"/>
+    <tableColumn id="5" name="due_date"/>
+    <tableColumn id="6" name="status"/>
+    <tableColumn id="7" name="verification_evidence"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium4" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="Reconciliation" displayName="Reconciliation" ref="A1:M6" headerRowCount="1">
   <autoFilter ref="A1:M6"/>
   <tableColumns count="13">
     <tableColumn id="1" name="reconciliation_id"/>
@@ -1379,7 +1398,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R3"/>
+  <dimension ref="A1:S3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1400,6 +1419,7 @@
     <col width="27" customWidth="1" min="16" max="16"/>
     <col width="42" customWidth="1" min="17" max="17"/>
     <col width="42" customWidth="1" min="18" max="18"/>
+    <col width="42" customWidth="1" min="19" max="19"/>
   </cols>
   <sheetData>
     <row r="1" ht="25" customHeight="1">
@@ -1493,6 +1513,11 @@
           <t>closed_duration_days</t>
         </is>
       </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>opened_week</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1573,6 +1598,10 @@
         <f>IF(G2&lt;&gt;"closed","",DATEVALUE(LEFT(P2,10))-DATEVALUE(LEFT(O2,10)))</f>
         <v/>
       </c>
+      <c r="S2">
+        <f>TEXT(DATEVALUE(LEFT(O2,10))-WEEKDAY(DATEVALUE(LEFT(O2,10)),2)+1,"yyyy-mm-dd")</f>
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1648,9 +1677,13 @@
         <f>IF(G3&lt;&gt;"closed","",DATEVALUE(LEFT(P3,10))-DATEVALUE(LEFT(O3,10)))</f>
         <v/>
       </c>
+      <c r="S3">
+        <f>TEXT(DATEVALUE(LEFT(O3,10))-WEEKDAY(DATEVALUE(LEFT(O3,10)),2)+1,"yyyy-mm-dd")</f>
+        <v/>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:R3"/>
+  <autoFilter ref="A1:S3"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -1659,6 +1692,132 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="42" customWidth="1" min="3" max="3"/>
+    <col width="35" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="23" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="25" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>action_id</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>case_id</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>process_change</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>owner</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>due_date</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>verification_evidence</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>ACTION-SYN-001</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>CASE-SYN-001</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Add a timestamped two-party handoff count and linked correction reason.</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Synthetic receiving process owner</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="n">
+        <v>46341</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>ACTION-SYN-002</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>CASE-SYN-002</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Request the synthetic correction log and handoff documentation.</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Synthetic inventory analyst</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>46331</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:G3"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2043,13 +2202,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:C10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -2166,13 +2325,12 @@
         </is>
       </c>
       <c r="B7" s="4">
-        <f>MEDIAN(Cases[closed_duration_days])</f>
-        <v/>
-      </c>
-      <c r="C7" s="4" t="inlineStr">
-        <is>
-          <t>Closed-case sample size: =COUNT(Cases[closed_duration_days])</t>
-        </is>
+        <f>IF(COUNT(Cases[closed_duration_days])=0,"",MEDIAN(Cases[closed_duration_days]))</f>
+        <v/>
+      </c>
+      <c r="C7" s="4">
+        <f>COUNT(Cases[closed_duration_days])</f>
+        <v/>
       </c>
     </row>
     <row r="8">
@@ -2181,36 +2339,51 @@
           <t>Action completion</t>
         </is>
       </c>
-      <c r="B8" s="4" t="inlineStr">
-        <is>
-          <t>Use COUNTIFS for verified completed and due actions</t>
-        </is>
+      <c r="B8" s="4">
+        <f>IFERROR(COUNTIFS(Actions[due_date],"&gt;="&amp;DATE(YEAR(TODAY()),MONTH(TODAY()),1),Actions[due_date],"&lt;="&amp;TODAY(),Actions[status],"completed",Actions[verification_evidence],"&lt;&gt;")/COUNTIFS(Actions[due_date],"&gt;="&amp;DATE(YEAR(TODAY()),MONTH(TODAY()),1),Actions[due_date],"&lt;="&amp;TODAY()),"")</f>
+        <v/>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Leave blank if no actions were due; require verification evidence</t>
+          <t>Month-to-date due actions only; blank when none are due; require verification evidence</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
+          <t>Overdue actions</t>
+        </is>
+      </c>
+      <c r="B9" s="4">
+        <f>COUNTIFS(Actions[due_date],"&lt;"&amp;TODAY(),Actions[status],"&lt;&gt;completed")</f>
+        <v/>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>Open actions with a due date before today</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
           <t>Limitations</t>
         </is>
       </c>
-      <c r="B9" s="4" t="inlineStr">
+      <c r="B10" s="4" t="inlineStr">
         <is>
           <t>Synthetic records; one closed-case example</t>
         </is>
       </c>
-      <c r="C9" s="4" t="inlineStr">
+      <c r="C10" s="4" t="inlineStr">
         <is>
           <t>Hashes do not prove authenticity; application audit is not immutable</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C9"/>
+  <autoFilter ref="A1:C10"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>